<commit_message>
📊 BIST Screener | 11.05.2026 16:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-11.xlsx
+++ b/data/bist_screener_2026-05-11.xlsx
@@ -3238,42 +3238,44 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>SNICA</t>
+          <t>KZBGY</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
-        <v>4.55</v>
+        <v>3.45</v>
       </c>
       <c r="C64" s="4" t="n">
-        <v>0.0089</v>
+        <v>0.0058</v>
       </c>
       <c r="D64" s="5" t="n">
-        <v>13350000</v>
+        <v>77780000</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>0.5366</v>
+        <v>0.348</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>74.13</v>
-      </c>
-      <c r="G64" s="2" t="inlineStr"/>
+        <v>54.63</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>17.31</v>
+      </c>
       <c r="H64" s="3" t="n">
         <v>0.57</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>-0.2148</v>
+        <v>0.038</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>-1.5579</v>
+        <v>-0.8970999999999999</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM TÜM, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr"/>
@@ -3281,44 +3283,42 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>MSGYO</t>
+          <t>SNICA</t>
         </is>
       </c>
       <c r="B65" s="7" t="n">
-        <v>6.58</v>
+        <v>4.55</v>
       </c>
       <c r="C65" s="8" t="n">
-        <v>-0.0266</v>
+        <v>0.0089</v>
       </c>
       <c r="D65" s="9" t="n">
-        <v>5190000</v>
+        <v>13350000</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>0.4424</v>
+        <v>0.5366</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>36.7</v>
-      </c>
-      <c r="G65" s="7" t="n">
-        <v>161.67</v>
-      </c>
+        <v>74.13</v>
+      </c>
+      <c r="G65" s="6" t="inlineStr"/>
       <c r="H65" s="7" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="I65" s="8" t="n">
-        <v>0.004099999999999999</v>
+        <v>-0.2148</v>
       </c>
       <c r="J65" s="8" t="n">
-        <v>-2.9577</v>
+        <v>-1.5579</v>
       </c>
       <c r="K65" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L65" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM TÜM, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M65" s="6" t="inlineStr"/>
@@ -3326,34 +3326,36 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AVPGY</t>
+          <t>MSGYO</t>
         </is>
       </c>
       <c r="B66" s="3" t="n">
-        <v>65.40000000000001</v>
+        <v>6.58</v>
       </c>
       <c r="C66" s="4" t="n">
-        <v>0.0243</v>
+        <v>-0.0266</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>1270000</v>
+        <v>5190000</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>0.2632</v>
+        <v>0.4424</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>79.73</v>
+        <v>36.7</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>13.27</v>
+        <v>161.67</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>0.0496</v>
-      </c>
-      <c r="J66" s="2" t="inlineStr"/>
+        <v>0.004099999999999999</v>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>-2.9577</v>
+      </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -3361,7 +3363,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr"/>
@@ -3369,40 +3371,42 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>TSPOR</t>
+          <t>AVPGY</t>
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>1.02</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="C67" s="8" t="n">
-        <v>0.02</v>
+        <v>0.0243</v>
       </c>
       <c r="D67" s="9" t="n">
-        <v>299170000</v>
+        <v>1270000</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>0.49</v>
+        <v>0.2632</v>
       </c>
       <c r="F67" s="7" t="n">
-        <v>55.87</v>
-      </c>
-      <c r="G67" s="6" t="inlineStr"/>
+        <v>79.73</v>
+      </c>
+      <c r="G67" s="7" t="n">
+        <v>13.27</v>
+      </c>
       <c r="H67" s="7" t="n">
         <v>0.59</v>
       </c>
       <c r="I67" s="8" t="n">
-        <v>-0.1067</v>
+        <v>0.0496</v>
       </c>
       <c r="J67" s="6" t="inlineStr"/>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M67" s="6" t="inlineStr"/>
@@ -3410,42 +3414,40 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>KOCMT</t>
+          <t>TSPOR</t>
         </is>
       </c>
       <c r="B68" s="3" t="n">
-        <v>2.8</v>
+        <v>1.02</v>
       </c>
       <c r="C68" s="4" t="n">
-        <v>0.0219</v>
+        <v>0.02</v>
       </c>
       <c r="D68" s="5" t="n">
-        <v>35720000</v>
+        <v>299170000</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0.2582</v>
+        <v>0.49</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>68.04000000000001</v>
+        <v>55.87</v>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
       <c r="H68" s="3" t="n">
         <v>0.59</v>
       </c>
       <c r="I68" s="4" t="n">
-        <v>-0.0862</v>
-      </c>
-      <c r="J68" s="4" t="n">
-        <v>-114.5083</v>
-      </c>
+        <v>-0.1067</v>
+      </c>
+      <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M68" s="2" t="inlineStr"/>
@@ -3453,42 +3455,42 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>YATAS</t>
+          <t>KOCMT</t>
         </is>
       </c>
       <c r="B69" s="7" t="n">
-        <v>44.06</v>
+        <v>2.8</v>
       </c>
       <c r="C69" s="8" t="n">
-        <v>-0.09970000000000001</v>
+        <v>0.0219</v>
       </c>
       <c r="D69" s="9" t="n">
-        <v>2130000</v>
+        <v>35720000</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>0.7472</v>
+        <v>0.2582</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>48.26</v>
-      </c>
-      <c r="G69" s="7" t="n">
-        <v>51.73</v>
-      </c>
+        <v>68.04000000000001</v>
+      </c>
+      <c r="G69" s="6" t="inlineStr"/>
       <c r="H69" s="7" t="n">
         <v>0.59</v>
       </c>
       <c r="I69" s="8" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="J69" s="6" t="inlineStr"/>
+        <v>-0.0862</v>
+      </c>
+      <c r="J69" s="8" t="n">
+        <v>-114.5083</v>
+      </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM TÜM, BIST ANA, BIST KAYSERİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST HALKA ARZ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M69" s="6" t="inlineStr"/>
@@ -3496,42 +3498,42 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ALARK</t>
+          <t>YATAS</t>
         </is>
       </c>
       <c r="B70" s="3" t="n">
-        <v>100.9</v>
+        <v>44.06</v>
       </c>
       <c r="C70" s="4" t="n">
-        <v>0.0177</v>
+        <v>-0.09970000000000001</v>
       </c>
       <c r="D70" s="5" t="n">
-        <v>6920000</v>
+        <v>2130000</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>0.3221</v>
+        <v>0.7472</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>63.18</v>
-      </c>
-      <c r="G70" s="2" t="inlineStr"/>
+        <v>48.26</v>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>51.73</v>
+      </c>
       <c r="H70" s="3" t="n">
         <v>0.59</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>-0.0125</v>
-      </c>
-      <c r="J70" s="4" t="n">
-        <v>-1.2814</v>
-      </c>
+        <v>0.013</v>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM TÜM, BIST ANA, BIST KAYSERİ</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr"/>
@@ -3539,42 +3541,42 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>AYEN</t>
+          <t>ALARK</t>
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>37</v>
+        <v>100.9</v>
       </c>
       <c r="C71" s="8" t="n">
-        <v>0.0238</v>
+        <v>0.0177</v>
       </c>
       <c r="D71" s="9" t="n">
-        <v>3060000</v>
+        <v>6920000</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>0.1697</v>
+        <v>0.3221</v>
       </c>
       <c r="F71" s="7" t="n">
-        <v>61.61</v>
-      </c>
-      <c r="G71" s="7" t="n">
-        <v>47.79</v>
-      </c>
+        <v>63.18</v>
+      </c>
+      <c r="G71" s="6" t="inlineStr"/>
       <c r="H71" s="7" t="n">
         <v>0.59</v>
       </c>
       <c r="I71" s="8" t="n">
-        <v>0.0143</v>
-      </c>
-      <c r="J71" s="6" t="inlineStr"/>
+        <v>-0.0125</v>
+      </c>
+      <c r="J71" s="8" t="n">
+        <v>-1.2814</v>
+      </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST KAYSERİ, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M71" s="6" t="inlineStr"/>
@@ -3582,44 +3584,42 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>PSGYO</t>
+          <t>AYEN</t>
         </is>
       </c>
       <c r="B72" s="3" t="n">
-        <v>3.5</v>
+        <v>37</v>
       </c>
       <c r="C72" s="4" t="n">
-        <v>0.09720000000000001</v>
+        <v>0.0238</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>275080000</v>
+        <v>3060000</v>
       </c>
       <c r="E72" s="4" t="n">
-        <v>0.4281</v>
+        <v>0.1697</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>67.93000000000001</v>
+        <v>61.61</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>4.7</v>
+        <v>47.79</v>
       </c>
       <c r="H72" s="3" t="n">
         <v>0.59</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>0.1378</v>
-      </c>
-      <c r="J72" s="4" t="n">
-        <v>6.6184</v>
-      </c>
+        <v>0.0143</v>
+      </c>
+      <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST KAYSERİ, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr"/>
@@ -3627,33 +3627,35 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>SEGYO</t>
+          <t>PSGYO</t>
         </is>
       </c>
       <c r="B73" s="7" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="C73" s="8" t="n">
-        <v>0</v>
+        <v>0.09720000000000001</v>
       </c>
       <c r="D73" s="9" t="n">
-        <v>18120000</v>
+        <v>275080000</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>0.2445</v>
+        <v>0.4281</v>
       </c>
       <c r="F73" s="7" t="n">
-        <v>51.54</v>
-      </c>
-      <c r="G73" s="6" t="inlineStr"/>
+        <v>67.93000000000001</v>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>4.7</v>
+      </c>
       <c r="H73" s="7" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="I73" s="8" t="n">
-        <v>-0.2247</v>
+        <v>0.1378</v>
       </c>
       <c r="J73" s="8" t="n">
-        <v>0.5464</v>
+        <v>6.6184</v>
       </c>
       <c r="K73" s="6" t="inlineStr">
         <is>
@@ -3662,7 +3664,7 @@
       </c>
       <c r="L73" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M73" s="6" t="inlineStr"/>
@@ -3670,44 +3672,42 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>DOAS</t>
+          <t>SEGYO</t>
         </is>
       </c>
       <c r="B74" s="3" t="n">
-        <v>184.6</v>
+        <v>5</v>
       </c>
       <c r="C74" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0</v>
       </c>
       <c r="D74" s="5" t="n">
-        <v>1480000</v>
+        <v>18120000</v>
       </c>
       <c r="E74" s="4" t="n">
-        <v>0.395</v>
+        <v>0.2445</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>44.54</v>
-      </c>
-      <c r="G74" s="3" t="n">
-        <v>14</v>
-      </c>
+        <v>51.54</v>
+      </c>
+      <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="3" t="n">
         <v>0.6</v>
       </c>
       <c r="I74" s="4" t="n">
-        <v>0.0475</v>
+        <v>-0.2247</v>
       </c>
       <c r="J74" s="4" t="n">
-        <v>-1.9014</v>
+        <v>0.5464</v>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr"/>
@@ -3715,42 +3715,44 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PENGD</t>
+          <t>DOAS</t>
         </is>
       </c>
       <c r="B75" s="7" t="n">
-        <v>14.84</v>
+        <v>184.6</v>
       </c>
       <c r="C75" s="8" t="n">
-        <v>-0.01</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D75" s="9" t="n">
-        <v>21890000</v>
+        <v>1480000</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>0.7673000000000001</v>
+        <v>0.395</v>
       </c>
       <c r="F75" s="7" t="n">
-        <v>68.95999999999999</v>
-      </c>
-      <c r="G75" s="6" t="inlineStr"/>
+        <v>44.54</v>
+      </c>
+      <c r="G75" s="7" t="n">
+        <v>14</v>
+      </c>
       <c r="H75" s="7" t="n">
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="I75" s="8" t="n">
-        <v>-0.059</v>
+        <v>0.0475</v>
       </c>
       <c r="J75" s="8" t="n">
-        <v>-2.8382</v>
+        <v>-1.9014</v>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST BURSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M75" s="6" t="inlineStr"/>
@@ -3758,44 +3760,42 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>SISE</t>
+          <t>PENGD</t>
         </is>
       </c>
       <c r="B76" s="3" t="n">
-        <v>52.35</v>
+        <v>14.84</v>
       </c>
       <c r="C76" s="4" t="n">
-        <v>0.0106</v>
+        <v>-0.01</v>
       </c>
       <c r="D76" s="5" t="n">
-        <v>91880000</v>
+        <v>21890000</v>
       </c>
       <c r="E76" s="4" t="n">
-        <v>0.4034</v>
+        <v>0.7673000000000001</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>66.72</v>
-      </c>
-      <c r="G76" s="3" t="n">
-        <v>13.97</v>
-      </c>
+        <v>68.95999999999999</v>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="3" t="n">
         <v>0.61</v>
       </c>
       <c r="I76" s="4" t="n">
-        <v>0.044</v>
+        <v>-0.059</v>
       </c>
       <c r="J76" s="4" t="n">
-        <v>-0.5445</v>
+        <v>-2.8382</v>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST BURSA</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr"/>
@@ -3803,42 +3803,44 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>ENTRA</t>
+          <t>SISE</t>
         </is>
       </c>
       <c r="B77" s="7" t="n">
-        <v>11.71</v>
+        <v>52.35</v>
       </c>
       <c r="C77" s="8" t="n">
-        <v>0.0272</v>
+        <v>0.0106</v>
       </c>
       <c r="D77" s="9" t="n">
-        <v>20750000</v>
+        <v>91880000</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>0.1936</v>
+        <v>0.4034</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>59.17</v>
-      </c>
-      <c r="G77" s="6" t="inlineStr"/>
+        <v>66.72</v>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>13.97</v>
+      </c>
       <c r="H77" s="7" t="n">
         <v>0.61</v>
       </c>
       <c r="I77" s="8" t="n">
-        <v>-0.0568</v>
+        <v>0.044</v>
       </c>
       <c r="J77" s="8" t="n">
-        <v>-24.3409</v>
+        <v>-0.5445</v>
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST ANKARA</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M77" s="6" t="inlineStr"/>
@@ -3846,44 +3848,42 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>EKGYO</t>
+          <t>ENTRA</t>
         </is>
       </c>
       <c r="B78" s="3" t="n">
-        <v>22.24</v>
+        <v>11.71</v>
       </c>
       <c r="C78" s="4" t="n">
-        <v>0.0109</v>
+        <v>0.0272</v>
       </c>
       <c r="D78" s="5" t="n">
-        <v>111260000</v>
+        <v>20750000</v>
       </c>
       <c r="E78" s="4" t="n">
-        <v>0.5065999999999999</v>
+        <v>0.1936</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>60.13</v>
-      </c>
-      <c r="G78" s="3" t="n">
-        <v>17.28</v>
-      </c>
+        <v>59.17</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="3" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="I78" s="4" t="n">
-        <v>0.0452</v>
+        <v>-0.0568</v>
       </c>
       <c r="J78" s="4" t="n">
-        <v>-23.3157</v>
+        <v>-24.3409</v>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST GAYRİMENKUL YO, BIST 50, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST KATILIM 50, BIST KATILIM 30, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST YILDIZ, BIST ANKARA</t>
         </is>
       </c>
       <c r="M78" s="2" t="inlineStr"/>
@@ -3891,38 +3891,44 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>TUKAS</t>
+          <t>EKGYO</t>
         </is>
       </c>
       <c r="B79" s="7" t="n">
-        <v>2.69</v>
+        <v>22.24</v>
       </c>
       <c r="C79" s="8" t="n">
-        <v>0.0189</v>
+        <v>0.0109</v>
       </c>
       <c r="D79" s="9" t="n">
-        <v>257300000</v>
+        <v>111260000</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>0.5413</v>
+        <v>0.5065999999999999</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>64.59</v>
-      </c>
-      <c r="G79" s="6" t="inlineStr"/>
+        <v>60.13</v>
+      </c>
+      <c r="G79" s="7" t="n">
+        <v>17.28</v>
+      </c>
       <c r="H79" s="7" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="I79" s="6" t="inlineStr"/>
-      <c r="J79" s="6" t="inlineStr"/>
+        <v>0.62</v>
+      </c>
+      <c r="I79" s="8" t="n">
+        <v>0.0452</v>
+      </c>
+      <c r="J79" s="8" t="n">
+        <v>-23.3157</v>
+      </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L79" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST İZMİR, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST GAYRİMENKUL YO, BIST 50, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST KATILIM 50, BIST KATILIM 30, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M79" s="6" t="inlineStr"/>
@@ -3930,40 +3936,38 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ISSEN</t>
+          <t>TUKAS</t>
         </is>
       </c>
       <c r="B80" s="3" t="n">
-        <v>8.710000000000001</v>
+        <v>2.69</v>
       </c>
       <c r="C80" s="4" t="n">
-        <v>0.0046</v>
+        <v>0.0189</v>
       </c>
       <c r="D80" s="5" t="n">
-        <v>1650000</v>
+        <v>257300000</v>
       </c>
       <c r="E80" s="4" t="n">
-        <v>0.2144</v>
+        <v>0.5413</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>65.94</v>
+        <v>64.59</v>
       </c>
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="3" t="n">
         <v>0.63</v>
       </c>
-      <c r="I80" s="4" t="n">
-        <v>-0.07629999999999999</v>
-      </c>
+      <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, BIST BALIKESİR</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST İZMİR, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr"/>
@@ -3971,42 +3975,40 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>KZBGY</t>
+          <t>ISSEN</t>
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>3.45</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="C81" s="8" t="n">
-        <v>0.0058</v>
+        <v>0.0046</v>
       </c>
       <c r="D81" s="9" t="n">
-        <v>77780000</v>
+        <v>1650000</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0.348</v>
+        <v>0.2144</v>
       </c>
       <c r="F81" s="7" t="n">
-        <v>54.63</v>
-      </c>
-      <c r="G81" s="7" t="n">
-        <v>16.67</v>
-      </c>
+        <v>65.94</v>
+      </c>
+      <c r="G81" s="6" t="inlineStr"/>
       <c r="H81" s="7" t="n">
         <v>0.63</v>
       </c>
       <c r="I81" s="8" t="n">
-        <v>0.0435</v>
+        <v>-0.07629999999999999</v>
       </c>
       <c r="J81" s="6" t="inlineStr"/>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, BIST BALIKESİR</t>
         </is>
       </c>
       <c r="M81" s="6" t="inlineStr"/>
@@ -14769,42 +14771,42 @@
     <row r="329">
       <c r="A329" s="6" t="inlineStr">
         <is>
-          <t>SOKE</t>
+          <t>ADGYO</t>
         </is>
       </c>
       <c r="B329" s="7" t="n">
-        <v>20.4</v>
+        <v>60.6</v>
       </c>
       <c r="C329" s="8" t="n">
-        <v>0</v>
+        <v>-0.0226</v>
       </c>
       <c r="D329" s="9" t="n">
-        <v>5960000</v>
+        <v>1530000</v>
       </c>
       <c r="E329" s="8" t="n">
-        <v>0.2451</v>
+        <v>0.2111</v>
       </c>
       <c r="F329" s="7" t="n">
-        <v>75.04000000000001</v>
+        <v>54.02</v>
       </c>
       <c r="G329" s="6" t="inlineStr"/>
       <c r="H329" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="I329" s="8" t="n">
-        <v>-0.0689</v>
+        <v>-0.06559999999999999</v>
       </c>
       <c r="J329" s="8" t="n">
-        <v>0.3541</v>
+        <v>0.8578</v>
       </c>
       <c r="K329" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L329" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST AYDIN</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M329" s="6" t="inlineStr"/>
@@ -14812,44 +14814,42 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>ISMEN</t>
+          <t>SOKE</t>
         </is>
       </c>
       <c r="B330" s="3" t="n">
-        <v>43.18</v>
+        <v>20.4</v>
       </c>
       <c r="C330" s="4" t="n">
-        <v>0.0179</v>
+        <v>0</v>
       </c>
       <c r="D330" s="5" t="n">
-        <v>9270000</v>
+        <v>5960000</v>
       </c>
       <c r="E330" s="4" t="n">
-        <v>0.3426</v>
+        <v>0.2451</v>
       </c>
       <c r="F330" s="3" t="n">
-        <v>50.12</v>
-      </c>
-      <c r="G330" s="3" t="n">
-        <v>9.06</v>
-      </c>
+        <v>75.04000000000001</v>
+      </c>
+      <c r="G330" s="2" t="inlineStr"/>
       <c r="H330" s="3" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="I330" s="4" t="n">
-        <v>0.2423</v>
+        <v>-0.0689</v>
       </c>
       <c r="J330" s="4" t="n">
-        <v>0.7472</v>
+        <v>0.3541</v>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA, BIST AYDIN</t>
         </is>
       </c>
       <c r="M330" s="2" t="inlineStr"/>
@@ -14857,42 +14857,44 @@
     <row r="331">
       <c r="A331" s="6" t="inlineStr">
         <is>
-          <t>KOTON</t>
+          <t>ISMEN</t>
         </is>
       </c>
       <c r="B331" s="7" t="n">
-        <v>16.18</v>
+        <v>43.18</v>
       </c>
       <c r="C331" s="8" t="n">
-        <v>0.0151</v>
+        <v>0.0179</v>
       </c>
       <c r="D331" s="9" t="n">
-        <v>3880000</v>
+        <v>9270000</v>
       </c>
       <c r="E331" s="8" t="n">
-        <v>0.1318</v>
+        <v>0.3426</v>
       </c>
       <c r="F331" s="7" t="n">
-        <v>64.53</v>
-      </c>
-      <c r="G331" s="6" t="inlineStr"/>
+        <v>50.12</v>
+      </c>
+      <c r="G331" s="7" t="n">
+        <v>9.06</v>
+      </c>
       <c r="H331" s="7" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
       <c r="I331" s="8" t="n">
-        <v>-0.1453</v>
+        <v>0.2423</v>
       </c>
       <c r="J331" s="8" t="n">
-        <v>-313.1914</v>
+        <v>0.7472</v>
       </c>
       <c r="K331" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L331" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M331" s="6" t="inlineStr"/>
@@ -14900,44 +14902,42 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>TRENJ</t>
+          <t>KOTON</t>
         </is>
       </c>
       <c r="B332" s="3" t="n">
-        <v>95.8</v>
+        <v>16.18</v>
       </c>
       <c r="C332" s="4" t="n">
-        <v>0.0424</v>
+        <v>0.0151</v>
       </c>
       <c r="D332" s="5" t="n">
-        <v>2320000</v>
+        <v>3880000</v>
       </c>
       <c r="E332" s="4" t="n">
-        <v>0.2848</v>
+        <v>0.1318</v>
       </c>
       <c r="F332" s="3" t="n">
-        <v>52.44</v>
-      </c>
-      <c r="G332" s="3" t="n">
-        <v>110.03</v>
-      </c>
+        <v>64.53</v>
+      </c>
+      <c r="G332" s="2" t="inlineStr"/>
       <c r="H332" s="3" t="n">
         <v>2.01</v>
       </c>
       <c r="I332" s="4" t="n">
-        <v>0.0216</v>
+        <v>-0.1453</v>
       </c>
       <c r="J332" s="4" t="n">
-        <v>-1.4265</v>
+        <v>-313.1914</v>
       </c>
       <c r="K332" s="2" t="inlineStr">
         <is>
-          <t>Enerji mineralleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L332" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M332" s="2" t="inlineStr"/>
@@ -14945,44 +14945,44 @@
     <row r="333">
       <c r="A333" s="6" t="inlineStr">
         <is>
-          <t>TBORG</t>
+          <t>TRENJ</t>
         </is>
       </c>
       <c r="B333" s="7" t="n">
-        <v>148.4</v>
+        <v>95.8</v>
       </c>
       <c r="C333" s="8" t="n">
-        <v>0.004099999999999999</v>
+        <v>0.0424</v>
       </c>
       <c r="D333" s="9" t="n">
-        <v>179240</v>
+        <v>2320000</v>
       </c>
       <c r="E333" s="8" t="n">
-        <v>0.0501</v>
+        <v>0.2848</v>
       </c>
       <c r="F333" s="7" t="n">
-        <v>54.49</v>
+        <v>52.44</v>
       </c>
       <c r="G333" s="7" t="n">
-        <v>14.82</v>
+        <v>110.03</v>
       </c>
       <c r="H333" s="7" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="I333" s="8" t="n">
-        <v>0.157</v>
+        <v>0.0216</v>
       </c>
       <c r="J333" s="8" t="n">
-        <v>-1.2844</v>
+        <v>-1.4265</v>
       </c>
       <c r="K333" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Enerji mineralleri</t>
         </is>
       </c>
       <c r="L333" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST ANKARA</t>
         </is>
       </c>
       <c r="M333" s="6" t="inlineStr"/>
@@ -14990,44 +14990,44 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>TRMET</t>
+          <t>TBORG</t>
         </is>
       </c>
       <c r="B334" s="3" t="n">
-        <v>128.5</v>
+        <v>148.4</v>
       </c>
       <c r="C334" s="4" t="n">
-        <v>0.043</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="D334" s="5" t="n">
-        <v>5240000</v>
+        <v>179240</v>
       </c>
       <c r="E334" s="4" t="n">
-        <v>0.4775</v>
+        <v>0.0501</v>
       </c>
       <c r="F334" s="3" t="n">
-        <v>50.27</v>
+        <v>54.49</v>
       </c>
       <c r="G334" s="3" t="n">
-        <v>26.7</v>
+        <v>14.82</v>
       </c>
       <c r="H334" s="3" t="n">
         <v>2.03</v>
       </c>
       <c r="I334" s="4" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.157</v>
       </c>
       <c r="J334" s="4" t="n">
-        <v>-1.3787</v>
+        <v>-1.2844</v>
       </c>
       <c r="K334" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L334" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST 50-30, BIST ANKARA, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M334" s="2" t="inlineStr"/>
@@ -15035,42 +15035,44 @@
     <row r="335">
       <c r="A335" s="6" t="inlineStr">
         <is>
-          <t>KLYPV</t>
+          <t>TRMET</t>
         </is>
       </c>
       <c r="B335" s="7" t="n">
-        <v>66</v>
+        <v>128.5</v>
       </c>
       <c r="C335" s="8" t="n">
-        <v>0.0451</v>
+        <v>0.043</v>
       </c>
       <c r="D335" s="9" t="n">
-        <v>3390000</v>
+        <v>5240000</v>
       </c>
       <c r="E335" s="8" t="n">
-        <v>0.1126</v>
+        <v>0.4775</v>
       </c>
       <c r="F335" s="7" t="n">
-        <v>66.63</v>
-      </c>
-      <c r="G335" s="6" t="inlineStr"/>
+        <v>50.27</v>
+      </c>
+      <c r="G335" s="7" t="n">
+        <v>26.7</v>
+      </c>
       <c r="H335" s="7" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="I335" s="8" t="n">
-        <v>-0.06150000000000001</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="J335" s="8" t="n">
-        <v>-1.6584</v>
+        <v>-1.3787</v>
       </c>
       <c r="K335" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L335" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST YILDIZ, BIST ANKARA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST 50-30, BIST ANKARA, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10</t>
         </is>
       </c>
       <c r="M335" s="6" t="inlineStr"/>
@@ -15078,42 +15080,42 @@
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>ISYAT</t>
+          <t>KLYPV</t>
         </is>
       </c>
       <c r="B336" s="3" t="n">
-        <v>8.69</v>
+        <v>66</v>
       </c>
       <c r="C336" s="4" t="n">
-        <v>-0.008</v>
+        <v>0.0451</v>
       </c>
       <c r="D336" s="5" t="n">
-        <v>2960000</v>
+        <v>3390000</v>
       </c>
       <c r="E336" s="4" t="n">
-        <v>0.6434000000000001</v>
+        <v>0.1126</v>
       </c>
       <c r="F336" s="3" t="n">
-        <v>59.49</v>
-      </c>
-      <c r="G336" s="3" t="n">
-        <v>203.99</v>
-      </c>
+        <v>66.63</v>
+      </c>
+      <c r="G336" s="2" t="inlineStr"/>
       <c r="H336" s="3" t="n">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="I336" s="4" t="n">
-        <v>0.0114</v>
-      </c>
-      <c r="J336" s="2" t="inlineStr"/>
+        <v>-0.06150000000000001</v>
+      </c>
+      <c r="J336" s="4" t="n">
+        <v>-1.6584</v>
+      </c>
       <c r="K336" s="2" t="inlineStr">
         <is>
-          <t>Çeşitli Hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L336" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST YILDIZ, BIST ANKARA</t>
         </is>
       </c>
       <c r="M336" s="2" t="inlineStr"/>
@@ -15121,44 +15123,42 @@
     <row r="337">
       <c r="A337" s="6" t="inlineStr">
         <is>
-          <t>ALVES</t>
+          <t>ISYAT</t>
         </is>
       </c>
       <c r="B337" s="7" t="n">
-        <v>3.51</v>
+        <v>8.69</v>
       </c>
       <c r="C337" s="8" t="n">
-        <v>0.0293</v>
+        <v>-0.008</v>
       </c>
       <c r="D337" s="9" t="n">
-        <v>143670000</v>
+        <v>2960000</v>
       </c>
       <c r="E337" s="8" t="n">
-        <v>0.7247</v>
+        <v>0.6434000000000001</v>
       </c>
       <c r="F337" s="7" t="n">
-        <v>53.47</v>
+        <v>59.49</v>
       </c>
       <c r="G337" s="7" t="n">
-        <v>56.8</v>
+        <v>203.99</v>
       </c>
       <c r="H337" s="7" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="I337" s="8" t="n">
-        <v>0.04190000000000001</v>
-      </c>
-      <c r="J337" s="8" t="n">
-        <v>3.7407</v>
-      </c>
+        <v>0.0114</v>
+      </c>
+      <c r="J337" s="6" t="inlineStr"/>
       <c r="K337" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Çeşitli Hizmetler</t>
         </is>
       </c>
       <c r="L337" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M337" s="6" t="inlineStr"/>
@@ -15166,44 +15166,44 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>GESAN</t>
+          <t>ALVES</t>
         </is>
       </c>
       <c r="B338" s="3" t="n">
-        <v>61.35</v>
+        <v>3.51</v>
       </c>
       <c r="C338" s="4" t="n">
-        <v>-0.0008</v>
+        <v>0.0293</v>
       </c>
       <c r="D338" s="5" t="n">
-        <v>19940000</v>
+        <v>143670000</v>
       </c>
       <c r="E338" s="4" t="n">
-        <v>0.3082</v>
+        <v>0.7247</v>
       </c>
       <c r="F338" s="3" t="n">
-        <v>78.03</v>
+        <v>53.47</v>
       </c>
       <c r="G338" s="3" t="n">
-        <v>24.83</v>
+        <v>56.8</v>
       </c>
       <c r="H338" s="3" t="n">
         <v>2.07</v>
       </c>
       <c r="I338" s="4" t="n">
-        <v>0.09720000000000001</v>
+        <v>0.04190000000000001</v>
       </c>
       <c r="J338" s="4" t="n">
-        <v>-0.8568000000000001</v>
+        <v>3.7407</v>
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L338" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST ANKARA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST ANKARA</t>
         </is>
       </c>
       <c r="M338" s="2" t="inlineStr"/>
@@ -15211,44 +15211,44 @@
     <row r="339">
       <c r="A339" s="6" t="inlineStr">
         <is>
-          <t>FROTO</t>
+          <t>GESAN</t>
         </is>
       </c>
       <c r="B339" s="7" t="n">
-        <v>97</v>
+        <v>61.35</v>
       </c>
       <c r="C339" s="8" t="n">
-        <v>-0.0051</v>
+        <v>-0.0008</v>
       </c>
       <c r="D339" s="9" t="n">
-        <v>22490000</v>
+        <v>19940000</v>
       </c>
       <c r="E339" s="8" t="n">
-        <v>0.1789</v>
+        <v>0.3082</v>
       </c>
       <c r="F339" s="7" t="n">
-        <v>39.12</v>
+        <v>78.03</v>
       </c>
       <c r="G339" s="7" t="n">
-        <v>10.76</v>
+        <v>24.83</v>
       </c>
       <c r="H339" s="7" t="n">
         <v>2.07</v>
       </c>
       <c r="I339" s="8" t="n">
-        <v>0.2187</v>
+        <v>0.09720000000000001</v>
       </c>
       <c r="J339" s="8" t="n">
-        <v>-0.5268999999999999</v>
+        <v>-0.8568000000000001</v>
       </c>
       <c r="K339" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L339" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST METAL ESYA MAKİNA, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST ANKARA</t>
         </is>
       </c>
       <c r="M339" s="6" t="inlineStr"/>
@@ -15256,42 +15256,44 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>ADGYO</t>
+          <t>FROTO</t>
         </is>
       </c>
       <c r="B340" s="3" t="n">
-        <v>60.6</v>
+        <v>97</v>
       </c>
       <c r="C340" s="4" t="n">
-        <v>-0.0226</v>
+        <v>-0.0051</v>
       </c>
       <c r="D340" s="5" t="n">
-        <v>1530000</v>
+        <v>22490000</v>
       </c>
       <c r="E340" s="4" t="n">
-        <v>0.2111</v>
+        <v>0.1789</v>
       </c>
       <c r="F340" s="3" t="n">
-        <v>54.02</v>
-      </c>
-      <c r="G340" s="2" t="inlineStr"/>
+        <v>39.12</v>
+      </c>
+      <c r="G340" s="3" t="n">
+        <v>10.76</v>
+      </c>
       <c r="H340" s="3" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="I340" s="4" t="n">
-        <v>-0.06559999999999999</v>
+        <v>0.2187</v>
       </c>
       <c r="J340" s="4" t="n">
-        <v>0.8578</v>
+        <v>-0.5268999999999999</v>
       </c>
       <c r="K340" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L340" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST YILDIZ</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST METAL ESYA MAKİNA, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M340" s="2" t="inlineStr"/>
@@ -25872,21 +25874,23 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>2.99</v>
+        <v>6.11</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0275</v>
+        <v>-0.0302</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>195360000</v>
-      </c>
-      <c r="E586" s="2" t="inlineStr"/>
+        <v>48320000</v>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F586" s="3" t="n">
-        <v>57.65</v>
+        <v>68.14</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25899,7 +25903,7 @@
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25907,42 +25911,40 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>17.8</v>
+        <v>152.2</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0114</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>16680000</v>
+        <v>1130000</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.9246</v>
+        <v>0.1071</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>54.39</v>
-      </c>
-      <c r="G587" s="7" t="n">
-        <v>168.24</v>
-      </c>
+        <v>54.75</v>
+      </c>
+      <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="8" t="n">
-        <v>0.0028</v>
+        <v>-3.6635</v>
       </c>
       <c r="J587" s="8" t="n">
-        <v>-10.3171</v>
+        <v>-0.4897</v>
       </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25950,21 +25952,21 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>6.16</v>
+        <v>18.71</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0016</v>
+        <v>0.0163</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>7070000</v>
+        <v>70370000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>60.92</v>
+        <v>59.18</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
@@ -25975,48 +25977,44 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L588" s="2" t="inlineStr"/>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>35.98</v>
+        <v>18.6</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0033</v>
+        <v>-0.0323</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>6120000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>64950000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>45.89</v>
-      </c>
-      <c r="G589" s="7" t="n">
-        <v>14.22</v>
-      </c>
+        <v>55.38</v>
+      </c>
+      <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26024,21 +26022,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>52.95</v>
+        <v>204.4</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0252</v>
+        <v>0.0089</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>19640000</v>
+        <v>11640000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>74.65000000000001</v>
+        <v>53.36</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26046,12 +26044,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26059,56 +26057,58 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>200.9</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0585</v>
+        <v>0.09140000000000001</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>7220000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>964780</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>70.69</v>
+        <v>62.64</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.004500000000000001</v>
+        <v>-0.0134</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>6460000</v>
+        <v>174500</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>66.33</v>
+        <v>11.61</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26116,53 +26116,43 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>2.71</v>
+        <v>15.02</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>30180000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>34230000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>44.63</v>
+        <v>62.91</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26170,23 +26160,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>6.11</v>
+        <v>36.66</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0302</v>
+        <v>-0.0043</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>48320000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>5380000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>68.14</v>
+        <v>65.25</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26194,12 +26182,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26207,69 +26195,81 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>81</v>
+        <v>21.12</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0134</v>
+        <v>0.0028</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>174500</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>793410</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>11.61</v>
+        <v>71.19</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L595" s="6" t="inlineStr"/>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>71.09999999999999</v>
+        <v>6.85</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.04559999999999999</v>
+        <v>-0.0228</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>897570</v>
+        <v>73070000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.1672</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>67.17</v>
+        <v>56.12</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
       <c r="J596" s="4" t="n">
-        <v>0.1431</v>
+        <v>-4.2562</v>
       </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26277,21 +26277,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>30.72</v>
+        <v>6.16</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0129</v>
+        <v>0.0016</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>26220000</v>
+        <v>7070000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>68.8</v>
+        <v>60.92</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26299,67 +26299,69 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>252.75</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0316</v>
+        <v>0.04559999999999999</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>9400</v>
+        <v>897570</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>51.88</v>
+        <v>67.17</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="J598" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>15.02</v>
+        <v>52.95</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.006</v>
+        <v>0.0252</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>34230000</v>
+        <v>19640000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>62.91</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26367,12 +26369,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26380,77 +26382,77 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>9.789999999999999</v>
+        <v>2.71</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.09140000000000001</v>
+        <v>0</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>964780</v>
+        <v>30180000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.95</v>
+        <v>0.7119</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>62.64</v>
+        <v>44.63</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="4" t="n">
-        <v>-23.6291</v>
+        <v>-191.6342</v>
       </c>
       <c r="J600" s="4" t="n">
-        <v>-0.4678</v>
+        <v>-0.8093</v>
       </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>21.12</v>
+        <v>31.18</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0028</v>
+        <v>0.0032</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>793410</v>
+        <v>14110000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.2667</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>71.19</v>
+        <v>60.07</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26458,104 +26460,88 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>78.65000000000001</v>
+        <v>45</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.06370000000000001</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>57710</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>6460000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>45.05</v>
+        <v>66.33</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J602" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
+      <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>36.66</v>
+        <v>80.8</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0043</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>5380000</v>
+        <v>10740000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>65.25</v>
+        <v>46.37</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="6" t="inlineStr"/>
       <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr">
-        <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+      <c r="K603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>6.85</v>
+        <v>19.42</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0228</v>
+        <v>-0.0147</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>73070000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>62740000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>56.12</v>
+        <v>38.21</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26563,7 +26549,7 @@
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26571,34 +26557,42 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>204.4</v>
+        <v>17.8</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0114</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>11640000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>16680000</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>53.36</v>
-      </c>
-      <c r="G605" s="6" t="inlineStr"/>
+        <v>54.39</v>
+      </c>
+      <c r="G605" s="7" t="n">
+        <v>168.24</v>
+      </c>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
+      <c r="I605" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J605" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26606,62 +26600,58 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>152.2</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.04099999999999999</v>
+        <v>-0.06370000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>1130000</v>
+        <v>57710</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.58</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>54.75</v>
+        <v>45.05</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="4" t="n">
-        <v>-3.6635</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J606" s="4" t="n">
-        <v>-0.4897</v>
+        <v>-4.155</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>19.42</v>
+        <v>30.72</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0147</v>
+        <v>-0.0129</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>62740000</v>
+        <v>26220000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>38.21</v>
+        <v>68.8</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26669,12 +26659,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26682,21 +26672,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>18.6</v>
+        <v>200.9</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0323</v>
+        <v>0.0585</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>64950000</v>
+        <v>7220000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>55.38</v>
+        <v>70.69</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26709,7 +26699,7 @@
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26717,21 +26707,23 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>18.71</v>
+        <v>252.75</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0163</v>
+        <v>-0.0316</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>70370000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>9400</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>59.18</v>
+        <v>51.88</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
@@ -26739,76 +26731,86 @@
       <c r="J609" s="6" t="inlineStr"/>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr"/>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>80.8</v>
+        <v>2.99</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.004099999999999999</v>
+        <v>0.0275</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>10740000</v>
+        <v>195360000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>46.37</v>
+        <v>57.65</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="2" t="inlineStr"/>
       <c r="J610" s="2" t="inlineStr"/>
-      <c r="K610" s="2" t="inlineStr"/>
-      <c r="L610" s="2" t="inlineStr"/>
+      <c r="K610" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>31.18</v>
+        <v>35.98</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0032</v>
+        <v>-0.0033</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>14110000</v>
+        <v>6120000</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.3528</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>60.07</v>
-      </c>
-      <c r="G611" s="6" t="inlineStr"/>
+        <v>45.89</v>
+      </c>
+      <c r="G611" s="7" t="n">
+        <v>14.22</v>
+      </c>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26835,7 +26837,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>11.05.2026 15:30</t>
+          <t>11.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 11.05.2026 17:33 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-11.xlsx
+++ b/data/bist_screener_2026-05-11.xlsx
@@ -25874,23 +25874,21 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>6.11</v>
+        <v>18.6</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0302</v>
+        <v>-0.0323</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>48320000</v>
-      </c>
-      <c r="E586" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>64950000</v>
+      </c>
+      <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>68.14</v>
+        <v>55.38</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25898,12 +25896,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25911,40 +25909,34 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>152.2</v>
+        <v>36.66</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.04099999999999999</v>
+        <v>-0.0043</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>1130000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>5380000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>54.75</v>
+        <v>65.25</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J587" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25952,56 +25944,48 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>18.71</v>
+        <v>80.8</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0163</v>
+        <v>-0.004099999999999999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>70370000</v>
+        <v>10740000</v>
       </c>
       <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>59.18</v>
+        <v>46.37</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K588" s="2" t="inlineStr"/>
+      <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>18.6</v>
+        <v>19.42</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0323</v>
+        <v>-0.0147</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>64950000</v>
+        <v>62740000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>55.38</v>
+        <v>38.21</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26009,12 +25993,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26022,21 +26006,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>204.4</v>
+        <v>45</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0089</v>
+        <v>0.004500000000000001</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>11640000</v>
+        <v>6460000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>53.36</v>
+        <v>66.33</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26044,12 +26028,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,35 +26041,35 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>9.789999999999999</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.09140000000000001</v>
+        <v>-0.06370000000000001</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>964780</v>
+        <v>57710</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.95</v>
+        <v>0.58</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>62.64</v>
+        <v>45.05</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-9.409700000000001</v>
       </c>
       <c r="J591" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-4.155</v>
       </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr"/>
@@ -26094,32 +26078,40 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>81</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0134</v>
+        <v>0.04559999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>174500</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>897570</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>11.61</v>
+        <v>67.17</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="J592" s="4" t="n">
+        <v>0.1431</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
@@ -26160,21 +26152,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>36.66</v>
+        <v>6.16</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0043</v>
+        <v>0.0016</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>5380000</v>
+        <v>7070000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>65.25</v>
+        <v>60.92</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26182,53 +26174,51 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>21.12</v>
+        <v>35.98</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0028</v>
+        <v>-0.0033</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>793410</v>
+        <v>6120000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.3528</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>71.19</v>
-      </c>
-      <c r="G595" s="6" t="inlineStr"/>
+        <v>45.89</v>
+      </c>
+      <c r="G595" s="7" t="n">
+        <v>14.22</v>
+      </c>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-0.2446</v>
+        <v>0.1029</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>0.3246</v>
+        <v>-1.4864</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26236,32 +26226,28 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.85</v>
+        <v>6.11</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0228</v>
+        <v>-0.0302</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>73070000</v>
+        <v>48320000</v>
       </c>
       <c r="E596" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.8667</v>
       </c>
       <c r="F596" s="3" t="n">
-        <v>56.12</v>
+        <v>68.14</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26269,7 +26255,7 @@
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26277,29 +26263,35 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>6.16</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.09140000000000001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>7070000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>964780</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>60.92</v>
+        <v>62.64</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L597" s="6" t="inlineStr"/>
@@ -26308,38 +26300,40 @@
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>71.09999999999999</v>
+        <v>2.71</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.04559999999999999</v>
+        <v>0</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>897570</v>
+        <v>30180000</v>
       </c>
       <c r="E598" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.7119</v>
       </c>
       <c r="F598" s="3" t="n">
-        <v>67.17</v>
+        <v>44.63</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
       <c r="J598" s="4" t="n">
-        <v>0.1431</v>
+        <v>-0.8093</v>
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26347,34 +26341,40 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>52.95</v>
+        <v>21.12</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0252</v>
+        <v>0.0028</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>19640000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>793410</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>74.65000000000001</v>
+        <v>71.19</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26382,40 +26382,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>2.71</v>
+        <v>18.71</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0</v>
+        <v>0.0163</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>30180000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>70370000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>44.63</v>
+        <v>59.18</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26423,23 +26417,23 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>31.18</v>
+        <v>252.75</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0032</v>
+        <v>-0.0316</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>14110000</v>
+        <v>9400</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.2667</v>
+        <v>0.2578</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>60.07</v>
+        <v>51.88</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26447,47 +26441,51 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>45</v>
+        <v>17.8</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.0114</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>6460000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>16680000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>66.33</v>
-      </c>
-      <c r="G602" s="2" t="inlineStr"/>
+        <v>54.39</v>
+      </c>
+      <c r="G602" s="3" t="n">
+        <v>168.24</v>
+      </c>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="2" t="inlineStr"/>
-      <c r="J602" s="2" t="inlineStr"/>
+      <c r="I602" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J602" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26495,48 +26493,62 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>80.8</v>
+        <v>152.2</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.004099999999999999</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>10740000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>1130000</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>46.37</v>
+        <v>54.75</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
-      <c r="K603" s="6" t="inlineStr"/>
-      <c r="L603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
+      <c r="K603" s="6" t="inlineStr">
+        <is>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>19.42</v>
+        <v>30.72</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0147</v>
+        <v>-0.0129</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>62740000</v>
+        <v>26220000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>38.21</v>
+        <v>68.8</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26544,12 +26556,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26557,42 +26569,34 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>17.8</v>
+        <v>204.4</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0114</v>
+        <v>0.0089</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>16680000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>11640000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>54.39</v>
-      </c>
-      <c r="G605" s="7" t="n">
-        <v>168.24</v>
-      </c>
+        <v>53.36</v>
+      </c>
+      <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26600,58 +26604,58 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>78.65000000000001</v>
+        <v>31.18</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.06370000000000001</v>
+        <v>0.0032</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>57710</v>
+        <v>14110000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.58</v>
+        <v>0.2667</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>45.05</v>
+        <v>60.07</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>30.72</v>
+        <v>200.9</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0129</v>
+        <v>0.0585</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>26220000</v>
+        <v>7220000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>68.8</v>
+        <v>70.69</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26659,12 +26663,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26672,21 +26676,21 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>200.9</v>
+        <v>2.99</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0585</v>
+        <v>0.0275</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>7220000</v>
+        <v>195360000</v>
       </c>
       <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>70.69</v>
+        <v>57.65</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
@@ -26694,12 +26698,12 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26707,54 +26711,62 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>252.75</v>
+        <v>6.85</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0228</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>9400</v>
+        <v>73070000</v>
       </c>
       <c r="E609" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.1672</v>
       </c>
       <c r="F609" s="7" t="n">
-        <v>51.88</v>
+        <v>56.12</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L609" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L609" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M609" s="6" t="inlineStr"/>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>2.99</v>
+        <v>81</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0275</v>
+        <v>-0.0134</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>195360000</v>
+        <v>174500</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>57.65</v>
+        <v>11.61</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26765,52 +26777,40 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>35.98</v>
+        <v>52.95</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0033</v>
+        <v>0.0252</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>6120000</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>19640000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>45.89</v>
-      </c>
-      <c r="G611" s="7" t="n">
-        <v>14.22</v>
-      </c>
+        <v>74.65000000000001</v>
+      </c>
+      <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J611" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26837,7 +26837,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>11.05.2026 16:30</t>
+          <t>11.05.2026 17:33</t>
         </is>
       </c>
     </row>

</xml_diff>